<commit_message>
fixed references on BOM
</commit_message>
<xml_diff>
--- a/hardware/SGI_BOM_v1.0.xlsx
+++ b/hardware/SGI_BOM_v1.0.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10208"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ashto\Dev\SeniorDesign_SwanGanz\hardware\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nathan/Dev/464H/SeniorDesign_SwanGanz/hardware/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCB992E4-9BC3-4BD9-839A-7D255EF6193B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D4EF2A0-812F-CB4C-B646-58510E51D942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Full Bom" sheetId="1" r:id="rId1"/>
@@ -79,48 +79,18 @@
     <t>R3</t>
   </si>
   <si>
-    <t>R4, R21, R22, R23, R24, R28, R29, R30, R35, R36, R37</t>
-  </si>
-  <si>
     <t>R5</t>
   </si>
   <si>
     <t>R6, R7, R8</t>
   </si>
   <si>
-    <t>R9, R13, R15, R17</t>
-  </si>
-  <si>
-    <t>R10, R14</t>
-  </si>
-  <si>
     <t>R11, R12</t>
   </si>
   <si>
-    <t>R16</t>
-  </si>
-  <si>
-    <t>R18</t>
-  </si>
-  <si>
-    <t>R19, R20</t>
-  </si>
-  <si>
-    <t>R25, R32</t>
-  </si>
-  <si>
-    <t>R26, R27, R33, R34</t>
-  </si>
-  <si>
-    <t>R31, R38</t>
-  </si>
-  <si>
     <t>SW1</t>
   </si>
   <si>
-    <t>SW2, SW2</t>
-  </si>
-  <si>
     <t>10k</t>
   </si>
   <si>
@@ -377,6 +347,36 @@
   </si>
   <si>
     <t>INA122UA/2K5</t>
+  </si>
+  <si>
+    <t>R10, R13</t>
+  </si>
+  <si>
+    <t>R15</t>
+  </si>
+  <si>
+    <t>SW2, SW3</t>
+  </si>
+  <si>
+    <t>R17</t>
+  </si>
+  <si>
+    <t>R18, R19</t>
+  </si>
+  <si>
+    <t>R9, R14, R16</t>
+  </si>
+  <si>
+    <t>R24, R31</t>
+  </si>
+  <si>
+    <t>R4,R20, R21, R22, R23, R27, R28, R29, R34, R35, R36</t>
+  </si>
+  <si>
+    <t>R25, R26, R32, R33</t>
+  </si>
+  <si>
+    <t>R30, R37</t>
   </si>
 </sst>
 </file>
@@ -448,21 +448,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -744,17 +741,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K23"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="47.81640625" customWidth="1"/>
-    <col min="2" max="2" width="20.08984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.08984375" customWidth="1"/>
-    <col min="4" max="4" width="22.90625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.36328125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="47.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.1640625" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -762,7 +759,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -786,103 +783,103 @@
         <v>11</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="C2" s="1">
         <v>14</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="I2" s="3">
         <v>0.05</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="K2" s="4">
         <v>0.1</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="C3" s="1">
         <v>1</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="E3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>42</v>
-      </c>
       <c r="H3" s="2" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="I3" s="3">
         <v>0.05</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="K3" s="4">
         <v>0.94</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="C4" s="1">
         <v>6</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="I4" s="3">
         <v>0.01</v>
@@ -894,24 +891,24 @@
         <v>0.91</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A5" s="10" t="s">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5" s="8" t="s">
         <v>13</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="C5" s="6">
+        <v>37</v>
+      </c>
+      <c r="C5" s="1">
         <v>3</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
@@ -919,537 +916,537 @@
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C6" s="6">
+        <v>41</v>
+      </c>
+      <c r="C6" s="1">
         <v>1</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>68</v>
+        <v>45</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>58</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="K6" s="4">
         <v>0.68</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C7" s="6">
+        <v>47</v>
+      </c>
+      <c r="C7" s="1">
         <v>2</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="I7" s="3">
         <v>0.01</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="K7" s="4">
         <v>0.1</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="C8" s="6">
+        <v>54</v>
+      </c>
+      <c r="C8" s="1">
         <v>1</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="I8" s="3">
         <v>0.01</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="K8" s="4">
         <v>0.25</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>17</v>
+        <v>114</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="C9" s="6">
+        <v>59</v>
+      </c>
+      <c r="C9" s="1">
         <v>11</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="I9" s="3">
         <v>0.01</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="K9" s="4">
         <v>0.11</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C10" s="6">
+        <v>65</v>
+      </c>
+      <c r="C10" s="1">
         <v>1</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="I10" s="3">
         <v>0.01</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="K10" s="4">
         <v>0.39</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="C11" s="6">
+        <v>69</v>
+      </c>
+      <c r="C11" s="1">
         <v>3</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="H11" s="8" t="s">
-        <v>108</v>
+        <v>74</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>98</v>
       </c>
       <c r="I11" s="3">
         <v>0.01</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="K11" s="4">
         <v>0.31</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>20</v>
+        <v>112</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="C12" s="6">
+        <v>73</v>
+      </c>
+      <c r="C12" s="1">
         <v>4</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="I12" s="3">
         <v>0.01</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="K12" s="4">
         <v>0.11</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>21</v>
+        <v>107</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C13" s="6">
+        <v>76</v>
+      </c>
+      <c r="C13" s="1">
         <v>2</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="F13" s="1">
         <v>100</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="I13" s="3">
         <v>0.01</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="K13" s="4">
         <v>0.1</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A14" s="10" t="s">
-        <v>22</v>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A14" s="8" t="s">
+        <v>19</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="C14" s="6">
+        <v>78</v>
+      </c>
+      <c r="C14" s="1">
         <v>2</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="F14" s="1">
         <v>0</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="K14" s="4">
         <v>0.21</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>23</v>
+        <v>108</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="C15" s="6">
+        <v>80</v>
+      </c>
+      <c r="C15" s="1">
         <v>1</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="I15" s="3">
         <v>0.01</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="K15" s="4">
         <v>0.1</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C16" s="1">
+        <v>1</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="C16" s="6">
-        <v>1</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="F16" s="1" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="I16" s="3">
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="K16" s="4">
         <v>0.1</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>25</v>
+        <v>111</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="C17" s="6">
+        <v>86</v>
+      </c>
+      <c r="C17" s="1">
         <v>2</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="F17" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H17" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>108</v>
       </c>
       <c r="I17" s="3">
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="K17" s="4">
         <v>0.11</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>26</v>
+        <v>113</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="C18" s="6">
+        <v>89</v>
+      </c>
+      <c r="C18" s="1">
         <v>2</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="F18" s="1">
         <v>200</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="I18" s="3">
         <v>0.01</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="K18" s="4">
         <v>0.12</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>27</v>
+        <v>115</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="C19" s="6">
+        <v>92</v>
+      </c>
+      <c r="C19" s="1">
         <v>4</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="I19" s="3">
         <v>0.01</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="K19" s="4">
         <v>0.1</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A20" s="9" t="s">
-        <v>28</v>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A20" s="7" t="s">
+        <v>116</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C20" s="6">
+        <v>96</v>
+      </c>
+      <c r="C20" s="1">
         <v>2</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="I20" s="3">
         <v>0.01</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="K20" s="4">
         <v>0.1</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="B21" s="1"/>
-      <c r="C21" s="6">
+      <c r="C21" s="1">
         <v>1</v>
       </c>
       <c r="D21" s="1"/>
@@ -1461,12 +1458,12 @@
       <c r="J21" s="1"/>
       <c r="K21" s="1"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>30</v>
+        <v>109</v>
       </c>
       <c r="B22" s="1"/>
-      <c r="C22" s="6">
+      <c r="C22" s="1">
         <v>2</v>
       </c>
       <c r="D22" s="1"/>
@@ -1478,38 +1475,38 @@
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A23" s="6" t="s">
-        <v>111</v>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A23" s="1" t="s">
+        <v>101</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="C23" s="6">
+        <v>106</v>
+      </c>
+      <c r="C23" s="1">
         <v>3</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="E23" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="F23" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="G23" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="H23" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="I23" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="J23" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="K23" s="11">
+        <v>102</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="J23" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="K23" s="4">
         <v>6.72</v>
       </c>
     </row>
@@ -1525,7 +1522,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96BDB06D-0379-43EC-B9E5-64348F2279C4}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>